<commit_message>
Update SSCUI data and add new files
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Temp/20260622_134619/sscui_export.xlsx
+++ b/Temp/20260622_134619/sscui_export.xlsx
@@ -10683,4 +10683,10 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{ea60d57e-af5b-4752-ac57-3e4f28ca11dc}" enabled="1" method="Standard" siteId="{36da45f1-dd2c-4d1f-af13-5abe46b99921}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>